<commit_message>
single file build script
</commit_message>
<xml_diff>
--- a/Excel/14_Electricity_Scope2_WIP_v01.xlsx
+++ b/Excel/14_Electricity_Scope2_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769B8BFE-7386-4B52-B58C-6B643923F71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2369FFCD-7FA9-4A2D-9B19-9DAF03C34601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Input - Electricity" sheetId="70" r:id="rId5"/>
     <sheet name="14.1.1-2 Purchased electricity" sheetId="69" r:id="rId6"/>
     <sheet name="Constants - Electricity" sheetId="110" r:id="rId7"/>
-    <sheet name="Constants - Common" sheetId="124" r:id="rId8"/>
+    <sheet name="Constants - Common" sheetId="125" r:id="rId8"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId9"/>
@@ -5513,16 +5513,16 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D81F84D6-5F02-4235-A746-BA8FE14805AF}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{0EB1895C-9E8C-4AF2-9E00-D6B27B0AC47D}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B7BF5B5E-79E0-4375-9D6A-D9FA1CCC4BF0}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{01803246-E4E7-4C12-9CED-FFEFC9C0B63F}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EF620D25-82C4-4E3D-903B-00DF550A6EC1}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{5C807759-03A6-4EA9-A3A8-2AE252F48040}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5531,7 +5531,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{09C2E716-989B-44D6-8205-F586D845F28C}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{511B8BA5-AF9B-4E90-8B77-F474961E5353}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5539,16 +5539,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0E0FF0E2-4620-43C1-9652-6882DCC167B3}" name="Temperature Zone">
+    <tableColumn id="1" xr3:uid="{BDF12359-4A77-42FA-90A4-CD462B7A32D5}" name="Temperature Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EBB63555-D964-49E1-A93F-50CDC1ED9AF9}" name="MAT">
+    <tableColumn id="2" xr3:uid="{05821D49-3078-4C26-8CEF-1FF0B81C6838}" name="MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A61AD894-ED82-4120-A8DE-AAECE008077D}" name="Min MAT">
+    <tableColumn id="3" xr3:uid="{85F0EB47-3E26-4081-A01B-790F8F5CC68D}" name="Min MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D6CE810E-80EC-4EFF-9F12-7F3D8D1492D9}" name="Max MAT">
+    <tableColumn id="4" xr3:uid="{A23E9FF0-621A-46DB-AF37-618721632CEB}" name="Max MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5557,7 +5557,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{665D01D1-7D41-4613-B144-A2AD51DBCEAD}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{FF9DBA8C-B8CD-451B-B149-E05E843AADC7}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5565,16 +5565,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C1ABE652-56A5-4FCD-910D-71EAAFFE6272}" name="Rainfall Zone">
+    <tableColumn id="1" xr3:uid="{B40E371A-E30C-4D44-9493-C4F0EC94E5A2}" name="Rainfall Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{01F34771-95FC-459D-90EE-E34410B3F51A}" name="Annual rainfall">
+    <tableColumn id="2" xr3:uid="{779E8154-16A3-4D17-86C3-715AC14DE8F0}" name="Annual rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2367FD5A-F217-4E81-8FA7-9CA50E5B32CA}" name="Min rainfall">
+    <tableColumn id="3" xr3:uid="{27F5D161-20D8-4A2C-B622-9C1ED7C8161C}" name="Min rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{6A975C09-C87C-4354-9534-7D8E89ED2691}" name="Max rainfall">
+    <tableColumn id="4" xr3:uid="{B7EF2610-84CC-454C-ADE9-87A434852E68}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5583,16 +5583,16 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{CBA1633D-76A7-4371-A04B-7BEABB0F08BB}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{5B4BE869-BD2D-4CB6-8F94-4C6FDFB0181F}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
   <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3069DED7-3874-48B1-B325-1C28269E9696}" name="Leaching Zone">
+    <tableColumn id="1" xr3:uid="{B6792D08-4CD9-4957-866D-CD24AC220047}" name="Leaching Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A25F4192-4944-4120-9915-82EF7025531E}" name="Leaching criteria">
+    <tableColumn id="2" xr3:uid="{4D8A101F-2F9D-48F4-9D0A-52C7A788BFA9}" name="Leaching criteria">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5601,16 +5601,16 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{FD5B05E3-19C6-4100-85DA-71098F8FF1CD}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{77B5BA89-C80A-47F2-A8B6-ED4B582A1C9C}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{9FC2C99A-B4B4-40F3-935D-925C300B8FDF}" name="Data source">
+    <tableColumn id="1" xr3:uid="{2F4FC8BB-B5E7-4221-86E1-4FA411077C77}" name="Data source">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D46139ED-F463-4707-8A4E-C41443E55E66}" name="Data score">
+    <tableColumn id="2" xr3:uid="{1CB283B2-6604-49C4-AD0B-13E9602B0421}" name="Data score">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5619,16 +5619,16 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{92A6190E-69B6-46CB-9191-620CC064B70A}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{2AEE2770-646A-43B3-B7B5-D9446C498E1F}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CEB4EA2B-5961-484D-8350-475743270E28}" name="Is in leaching zone">
+    <tableColumn id="1" xr3:uid="{F906496D-A444-4250-8922-433A11D3B881}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0CC4EA28-8CD5-41A6-B3AE-584D325AA33B}" name="FracWET" dataDxfId="19">
+    <tableColumn id="2" xr3:uid="{878DA8B7-C630-4AB9-8C95-90F444A5D738}" name="FracWET" dataDxfId="19">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5637,7 +5637,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{6679BB2F-3579-43A8-A109-831B9D7B54D8}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{5F2CF032-D7F2-4844-ACBE-EFAB422E543F}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5646,19 +5646,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{4BA3F7B5-656F-45F8-BF3E-0A484F916F2F}" name="Production system j">
+    <tableColumn id="1" xr3:uid="{2D0807DD-6AA3-4428-AB95-96AA52AB5C1D}" name="Production system j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B90E68FC-CC79-4012-9A46-74590680DBD1}" name="EFN2O">
+    <tableColumn id="2" xr3:uid="{8FCA39AD-469E-4CD3-80A6-3C5099BC6238}" name="EFN2O">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3E21F76F-F5B2-4041-AAB1-F17D742FCD53}" name="Production system only">
+    <tableColumn id="3" xr3:uid="{7F5F1FED-030A-4162-A69C-E39984CC7BDC}" name="Production system only">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{39D51D26-A968-47F0-9E51-DC6A0F6E496F}" name="Irrigation method">
+    <tableColumn id="4" xr3:uid="{AAB52485-33EF-46FC-9F4B-36BDA871301C}" name="Irrigation method">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{617965C5-0EFE-4A87-944D-F7E1E324C50E}" name="Rainfall zone">
+    <tableColumn id="5" xr3:uid="{FF942727-9CF7-4E83-B62C-E3D00A8D558C}" name="Rainfall zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5667,16 +5667,16 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{43666865-6CB6-4F03-BDD0-3B6F4D323A26}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{082E5E6E-359C-40E3-A8D2-658EDE7A0FAC}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D36499D2-CCF3-46C5-BB72-A3F37BE9B792}" name="Irrigation type i">
+    <tableColumn id="1" xr3:uid="{6814AD1A-7016-44E0-9C99-03FF83468F83}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E58B17F5-7400-4903-9AB4-DD555181EBCE}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AFA1116F-C725-4B55-9B70-E01F18D7D64D}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5685,16 +5685,16 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{92BBB9E2-27EA-410F-94C6-6A9613891B1C}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{F5B896D3-D18E-4B82-B16D-832D4CAA1995}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{C9C04E5A-660E-414D-9DB6-01838B3492DB}" name="Climate zone">
+    <tableColumn id="1" xr3:uid="{A6E8A000-CB3A-4589-A633-510CB794A021}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3600E549-0C23-4C73-853F-38656552208F}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{91A37728-9D03-42EE-883F-34C68FDE0991}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5703,16 +5703,16 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{5864E18A-85D3-4273-9E20-4532030E26B3}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{84600146-C8D5-41EF-B31F-A7FCF6202E58}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{90AB03FE-8F25-4902-83AB-AD574E2AE79F}" name="Month">
+    <tableColumn id="1" xr3:uid="{873729FE-B0B8-43E5-88AE-8D20F76416C4}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B8AD1E96-22A5-41C3-A4A7-D7E6FE966E54}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{C4C2B80B-A079-4091-9A9A-9B58521D39CA}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5749,7 +5749,7 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{2D84D5F9-E8B5-4E78-90DA-0C63DDED5B62}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{DD97BDBB-20B1-4018-B059-7F2FC8F608C2}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5769,52 +5769,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{A01B4BA3-FD22-4670-BA5A-4B00002FF4CC}" name="Temperature zone">
+    <tableColumn id="1" xr3:uid="{DC67277F-0CDC-427E-9644-E5596A7F4494}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6A82FDF1-BD5A-407B-8304-815428D8B8D6}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{45D33B11-136F-44DC-920F-653DE287B84F}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16CD879-0333-4717-9686-07EB7DE1144B}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{B78AD67B-4603-44F8-AA5D-4C3A9CDD0A62}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{520B4E21-B08A-4C84-896B-179A1486D9A5}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{0583BDDD-1635-4862-BADC-97F1690AFE48}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{4EE05FD7-FB2B-4416-85FB-12E77FE265D7}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{F809273A-73C8-40D4-9C50-F2D5C93DEE56}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{842B5FAD-3960-48D2-AA76-2A14ED3A6477}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{00449008-A3E7-4114-B413-65EB97C892A9}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{81C5D01F-CFD3-4A31-9B91-D9D056C43FFB}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{2758521E-4AF2-4F97-9BD8-45186E981572}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{3D71210C-E282-491F-B729-EAE862599B9C}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{D0A95670-DDCD-45AC-9636-5330B17C3937}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5975C33C-D2BF-4942-A031-A4A2F7B4D7C9}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{F969F9D4-6A52-406A-879A-DB1CBD98D2A6}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BBB9A1AF-7EBC-4F25-8AB3-C74863606377}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{1131A76B-25CC-4D1D-ACF4-DE2010E0B5D0}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{DA20D397-931E-4699-BD22-1E411B451CC6}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{B570B9BE-F6E9-4755-A835-3AEDA6FE5D89}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{6CE558FB-0EB4-42FD-A611-9F95525E2DAE}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{290F1253-0E30-47CF-986A-587171B375E4}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DC8A560F-F38D-49F7-A98A-0ACDFDB241EB}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{B4AB0FB4-EB82-415D-9571-BA6462BBB4A8}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{D270B3DB-0434-4938-AB52-EA893908A250}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{A3CFDE98-4294-455E-B95C-7948165A6283}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{8AF12068-A0F7-483F-BD80-338F22D0E820}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{077C2B6B-A9ED-4CEF-A0D5-977191F456F7}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{FF15217F-2865-4B95-8A72-D06E4833856B}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{8B0D34FB-6534-4647-9CA2-FF689189ADC8}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5823,16 +5823,16 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{3CC6091B-B0E7-47DA-8A34-9E97385F83DA}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="38" xr:uid="{3777A1D9-9AB6-4A99-9843-98D8910F3861}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7BA53F75-A677-4CCA-AACA-FCBEAE0518DE}" name="Climate Zone">
+    <tableColumn id="1" xr3:uid="{90353079-6C94-4374-B3F7-E6CEFC89A25E}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8AC0609E-C2EF-49E1-BE29-0C6E25006CD5}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{62DF64D2-D979-40F8-9AB6-D16FDA4EAAAD}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5893,20 +5893,20 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9C895DF2-CA6E-4D0A-87E7-CCB379DADCA6}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2D45D258-076A-4B5A-AA6B-C49DFA191D56}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
   <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{8D613318-2B70-4670-B258-221EA9035D24}" name="State/Territory">
+    <tableColumn id="1" xr3:uid="{795177ED-1EBA-43C6-9498-92077FE04B20}" name="State/Territory">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{116E9D89-204F-4F01-919B-43912E7ED4E1}" name="Common Name">
+    <tableColumn id="2" xr3:uid="{E6772BFB-AA6A-41FC-BD6C-C9E793BB4773}" name="Common Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{31D770C2-E869-4A79-A451-0662C6E1CBCD}" name="Abbreviation">
+    <tableColumn id="3" xr3:uid="{F56D49FB-4059-499C-A541-DB617EE84BCF}" name="Abbreviation">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5915,12 +5915,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F746F6D8-5BBC-4885-921A-E95E96ADC256}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4AF5C838-87E8-4D7B-A7BB-621E19D72D16}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2DE85C96-DDB1-4045-9E68-7C60CDB31588}" name="SA 4 Name">
+    <tableColumn id="1" xr3:uid="{D87A9820-7D5C-4E3B-9FDA-0760A549099D}" name="SA 4 Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5929,16 +5929,16 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{DD857DC9-3D73-4790-86C2-F19A28F49DB7}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{6CEEA0DB-3426-4FC4-9C05-FC16BB4DB114}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5806787F-6760-4C3E-8A5E-2CF4567CE52B}" name="Gas">
+    <tableColumn id="1" xr3:uid="{449CE4B5-C92A-4D75-AD48-7B18A369707C}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{068169CF-D1E7-4746-9274-630DF775F444}" name="CO2-e factor">
+    <tableColumn id="2" xr3:uid="{6207AA7D-D9A5-4D47-B8E9-BAB69025D4FE}" name="CO2-e factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5947,7 +5947,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{5892552B-3207-434B-8574-F3A1732EC0CB}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{E4C15A35-8E09-4760-B0A3-618AB40690CB}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5956,19 +5956,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{76CD55DC-1E4F-4605-8D79-E77E89E3D021}" name="Gas">
+    <tableColumn id="1" xr3:uid="{C52D27CF-AD7B-42B7-B36E-CFB70CF6CB19}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{020278C9-0336-41BF-BA74-DBB91AB3F9F4}" name="Conversion factor">
+    <tableColumn id="5" xr3:uid="{303926E1-9540-448E-BD4A-87D980C3A4AC}" name="Conversion factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{57549EBF-D1CC-4F5C-9EA8-9537A829ADDA}" name="Conversion factor 1">
+    <tableColumn id="2" xr3:uid="{6B00D6B4-3A7A-40A7-8FDE-B4C76D5AE8B2}" name="Conversion factor 1">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{12FA7817-C6A8-4D44-ADA8-E81EEEDFA9BA}" name="Conversion factor 2">
+    <tableColumn id="3" xr3:uid="{E2935796-0188-45BB-81D5-45675D22D87B}" name="Conversion factor 2">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{C594A305-79A2-43FE-988F-8BBBB68DD811}" name="Conversion factor combined">
+    <tableColumn id="4" xr3:uid="{C129806A-705C-4D9D-807B-FDF830B070C7}" name="Conversion factor combined">
       <calculatedColumnFormula>Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 1]]/Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 2]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5977,7 +5977,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{B0EE78FA-AA91-4D59-9636-639333E81ACC}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{1DC25208-F11F-41FC-A971-293EC942CEA7}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -5997,52 +5997,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{B8163958-A5D7-432F-8169-74980C5E627E}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{70C65BBD-65EB-401C-841C-2F90C27F1229}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{76EAA88C-E07E-49B6-93F7-AE21CCDFCF85}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{04F52095-F2E8-4CFF-BC02-735327398AE7}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{56C8A0E9-257F-4581-ADBA-06A58F8CBC65}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{293C01F0-58C5-4225-B1BF-0AF76DD11236}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E4D32458-34A7-40AA-A1FC-2A577CB2729D}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{589D5993-98E6-4F10-8BEF-F4D3384D2A1A}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{985786B8-AFE1-496E-ADDB-128D77BEB255}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{406FCB98-F580-476B-8094-37A732C5209C}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{99284B7D-9D02-4BBC-8258-39B7339A5AE8}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{7AA1A242-2BD3-4A2A-9FF2-041A49F70FC5}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{2B1D0977-E9CB-465D-BDC5-3D8F7C67D669}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{FD90A26C-F6B4-4CA9-BFD9-37F32B561D34}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{2BF2EBCF-953A-45E3-BD68-3DCE245E2AD7}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{F2BE60C6-21D0-4D92-962B-F8714AA70957}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{0751C6A7-8EB7-4076-8C23-A33E75039F66}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{9483392B-977A-4443-87CA-3F71C94B91EE}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{0267D1FA-A900-4A6F-B28C-3F50EDFBB6EE}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{66A31397-B101-451A-AFF2-657EEC54BB8A}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{DD5F33D8-80FC-4F51-BD18-707285C96EF5}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{76E99937-B5E0-46CF-8F37-854ABC92A2CE}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{9CCB599B-58D4-4366-8A9B-C02110B0D6CB}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{79453B92-681F-4F2C-A55A-6A70BFA2A296}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{67C98518-B842-4FCF-94D5-843FEAE5E0E7}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{241623C7-2535-40B3-98B6-CB4E146DC870}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{952AACAA-D47D-4645-9869-B0900B82A660}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{01C0BA39-A5B7-4660-87AF-2141015EE601}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{8F001C74-AE11-4E37-BF8A-9A6762C22CAE}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{3B44E29E-E339-424C-9EF8-8294D5D9D33A}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{5691A2AB-CAA4-4666-BF1E-C36424D22BD7}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{376D0424-4DC1-4C50-81D5-DF1A20DAAAAB}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9908,7 +9908,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3566AFB0-B4A9-4456-8FA3-C3E6CEB44C48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{235791DA-4C9F-4E69-8908-19D0D65BC2E4}">
   <dimension ref="A1:BY259"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13900,6 +13900,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -14094,31 +14114,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACkAKgAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADIAKQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsACAARABlAGwAaQBtAGkAdABlAHIALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEAXQAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgBdACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgBYAE0ATAAoAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAHQAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAApACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAC8AdABcAHUAMAAwADMAZQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AG0AYQBwAF8AcABlAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAXAAiACAAdABvACAAXAAiACAAXAB1ADAAMAAyADYAIABlAG4AZABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAFwAdQAwADAAMwBlADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAdQAwADAAMgA3AFwAIgAgAFwAdQAwADAAMgA2ACAAcwBoACAAXAB1ADAAMAAyADYAIABcACIAXAB1ADAAMAAyADcAIQBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0AFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ASQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACkAIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAYQBzAHMAbwBjAGkAYQB0AGUAZAAgAHcAaQB0AGgAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGEAbgBkACAAbABvAHMAcwBlAHMAIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwAgAGwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAbABvAGMAYQB0AGkAbwBuAC0AYgBhAHMAZQBkACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGEAcwBzAG8AYwBpAGEAdABlAGQAIAB3AGkAdABoACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABhAG4AZAAgAGwAbwBzAHMAZQBzACAAbwBmACAAcAB1AHIAYwBoAGEAcwBlAGQAIABvAHIAIABhAGMAcQB1AGkAcgBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAAxAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALAAgAFQAZQByAHIAaQB0AG8AcgB5ACAAbwByACAAZwByAGkAZAAgAGQAZQBzAGMAcgBpAHAAdABpAG8AbgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAEMAVABcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIAAwAC4ANwA4ACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgADAALgA2ADcALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADAALgAyADIALAAgADAALgAwADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdAAgAEkAbgB0AGUAcgBjAG8AbgBuAGUAYwB0AGUAZAAgAFMAeQBzAHQAZQBtACAAKABTAFcASQBTACkAXAAiACwAIAAwAC4ANQAwACwAIAAwAC4AMAA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAZQByAG4AIABJAG4AdABlAHIAYwBvAG4AbgBlAGMAdABlAGQAIABTAHkAcwB0AGUAbQAgACgATgBXAEkAUwApAFwAIgAsACAAMAAuADUANgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgADAALgAyADAALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQAgAC0AIABEAGEAcgB3AGkAbgAgAEsAYQB0AGgAZQByAGkAbgBlACAASQBuAHQAZQByAGMAbwBuAG4AZQBjAHQAZQBkACAAUwB5AHMAdABlAG0AIAAoAEQASwBJAFMAKQBcACIALAAgADAALgA1ADYALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdABpAG8AbgBhAGwAXAAiACwAIAAwAC4ANgAyACwAIAAwAC4AMAA3AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATgBTAFcAIABhAG4AZAAgAEEAQwBUACAAcwBwAGwAaQB0ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAHIAbwB3AHMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBSAGUAcwBpAGQAdQBhAGwAIABNAGkAeAAgAEYAYQBjAHQAbwByACAAZgBvAHIAIABtAGEAcgBrAGUAdAAtAGIAYQBzAGUAZAAgAGUAcQB1AGEAdABpAG8AbgBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFQAYQBiAGwAZQAgADIAYQAgAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAcgBvAG0AIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQA6ACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABmAGEAYwB0AG8AcgBzACAAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADIAYQBcACIAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACwAIABUAGUAcgByAGkAdABvAHIAeQAgAG8AcgAgAGcAcgBpAGQAIABkAGUAcwBjAHIAaQBwAHQAaQBvAG4AXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAaQBvAG4AYQBsAFwAIgAsACAAMAAuADgAMQAsACAAMgAyADYALAAgADAALgAxADAALAAgADIAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQA0ADoAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEANAAuADEALgAxACAAUAB1AHIAYwBoAGEAcwBlAGQAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAAoAEwAbwBjAGEAdABpAG8AbgAtAEIAYQBzAGUAZAApAFwAbgAxADQALgAxAC4AMgAgAFAAdQByAGMAaABhAHMAZQBkACAARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABNAGEAcgBrAGUAdAAtAEIAYQBzAGUAZAApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcAG4ARQBfADIAZQBsAGUAYwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwB7ADIALABlAGwAZQBjAH0APQBRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAMgAsAGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4AUQBfAGUAbABlAGMAIAA9ACAAYQBtAG8AdQBuAHQAIABvAGYAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABwAHUAcgBjAGgAYQBzAGUAZAAgAGYAcgBvAG0AIAB0AGgAZQAgAGcAcgBpAGQAIAAoAGsAVwBoACkAXABuAEUARgBfADIAZQBsAGUAYwAgAD0AIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgACgAawBnACAAQwBPADIAZQAvAGsAVwBoACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAGUAbABlAGMALAAgAEUARgBfADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACAAKgAgAEUARgBfADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEANAAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAMgAsAGUAbABlAGMAfQA9AFEAXwB7AGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfADIAZQBsAGUAYwBcACIALAAgAFwAIgBsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIALAAgAFwAIgBrAGcAIABDAE8AMgBlAC8AawBXAGgAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGQAZABlAGQAIABnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYwBhAHAAdAB1AHIAZQAgAHcAaABpAGMAaAAgAGcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAE0AYQByAGsAZQB0AC0AYgBhAHMAZQBkACAAUwBjAG8AcABlACAAMgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHAAdQByAGMAaABhAHMAZQBkACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAbgBFAF8AMgBlAGwAZQBjAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAHsAMgAsAGUAbABlAGMAfQA9ACgAKABRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAKQAtACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBSAE0ARgAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBRAF8AZQBsAGUAYwAgAD0AIABhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZAAgACgAawBXAGgAKQBcAG4AUgBQAFAAIAA9ACAAUgBlAG4AZQB3AGEAYgBsAGUAIABQAG8AdwBlAHIAIABQAGUAcgBjAGUAbgB0AGEAZwBlACAAdQBuAGQAZQByACAAdABoAGUAIABMAGEAcgBnAGUALQBzAGMAYQBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAVABhAHIAZwBlAHQAIAAoAEwAUgBFAFQAKQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgBKAFIAUABQACAAPQAgAGoAdQByAGkAcwBkAGkAYwB0AGkAbwBuAGEAbAAgAHIAZQBuAGUAdwBhAGIAbABlACAAcABvAHcAZQByACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAG8AbgBsAHkAIABhAHAAcABsAGkAZQBzACAAdABvACAAdABoAGUAIABBAEMAVAApACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAFIARQBDAF8AbwBuAHMAaQB0AGUAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB0AGgAYQB0ACAAaABhAHYAZQAgAGIAZQBlAG4AIABvAHIAIAB3AGkAbABsACAAYgBlACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAEUARgBfAFIATQBGADIAZQBsAGUAYwAgAD0AIABTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABrAGcAIABDAE8AMgBlAC8AawBXAGgAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgAC0AMwApACkAIAAqACAARQBGAF8AUgBNAEYAMgBlAGwAZQBjACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgADMAKQApACAAKgAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcAB1AHIAYwBoAGEAcwBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADQALgAxAC4AMgAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewAyACwAZQBsAGUAYwB9AD0AKABRAF8AewBlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAKAAxAC0AKABSAFAAUAArAEoAUgBQAFAAKQApACAALQAgACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7ADIALABlAGwAZQBjAH0APQAoAFEAXwB7AGUAbABlAGMAfQAgAFwAXAB0AGkAbQBlAHMAIAAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAIAAtACAAKAAoAFIARQBDAF8AewBzAHUAcgByAGUAbgBkAGUAcgBlAGQAfQAtAFIARQBDAF8AewBvAG4AcwBpAHQAZQB9ACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsAMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAUABQAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAUABvAHcAZQByACAAUABlAHIAYwBlAG4AdABhAGcAZQAgAHUAbgBkAGUAcgAgAHQAaABlACAATABhAHIAZwBlAC0AcwBjAGEAbABlACAAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAFQAYQByAGcAZQB0ACAAKABMAFIARQBUACkAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBSAFAAUABcACIALAAgAFwAIgBqAHUAcgBpAHMAZABpAGMAdABpAG8AbgBhAGwAIAByAGUAbgBlAHcAYQBiAGwAZQAgAHAAbwB3AGUAcgAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABmAG8AcgAgAHQAaABlACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHAAZQByAGkAbwBkACAAKABBAEMAVAAgAG8AbgBsAHkAKQBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZABcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIARQBDAF8AbwBuAHMAaQB0AGUAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAEMAZQByAHQAaQBmAGkAYwBhAHQAZQBzACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAFIATQBGADIAZQBsAGUAYwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUALwBrAFcAaABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAASQBuACAAbwByAGQAZQByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAG0AZQBnAGEAdwBhAHQAdAAgAGgAbwB1AHIAcwAgAHQAbwAgAGsAaQBsAG8AdwBhAHQAdAAgAGgAbwB1AHIAcwAsACAAdABoAGUAIABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAGEAbgBkACAAUgBFAEMAXwBvAG4AcwBpAHQAZQAgAHYAYQByAGkAYQBiAGwAZQBzACAAYQByAGUAIABtAHUAbAB0AGkAcABsAGkAZQBkACAAYgB5ACAAMQAwAF4AMwAgAGkAbgBzAHQAZQBhAGQAIABvAGYAIAAxADAAXgAtADMALgBcACIAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBTAG8AdQByAGMAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAYQB0AGEAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVABpAHQAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAVgBhAHIAaQBhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14137,25 +14156,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>

</xml_diff>